<commit_message>
ecommerce: spell out concrete UI steps for FE/UI cases in TestCases.xlsx (screen, URL, navigation, on-screen check)
</commit_message>
<xml_diff>
--- a/testcases/TestCases.xlsx
+++ b/testcases/TestCases.xlsx
@@ -5602,7 +5602,9 @@
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue lists the active products, once each</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue lists the active products, once each.</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
@@ -5652,7 +5654,9 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>Then every catalogue price on screen equals the product row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: every catalogue price on screen equals the product row.</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
@@ -5702,7 +5706,9 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>Then product 6 is shown out of stock</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: product 6 is shown out of stock.</t>
         </is>
       </c>
       <c r="H99" s="3" t="inlineStr">
@@ -5752,7 +5758,9 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>Then product 1 is shown in stock</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: product 1 is shown in stock.</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
@@ -5802,7 +5810,9 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue does not list product 9</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue does not list product 9.</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr">
@@ -5852,8 +5862,10 @@
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 4 is opened
-Then the product page name, price and SKU equal row 4</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/4) — on the catalogue, click product 4.
+4. On screen, verify: the product page name, price and SKU equal row 4.</t>
         </is>
       </c>
       <c r="H102" s="3" t="inlineStr">
@@ -5903,8 +5915,10 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 2 is opened
-Then the product page stock equals row 2</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/2) — on the catalogue, click product 2.
+4. On screen, verify: the product page stock equals row 2.</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr">
@@ -5954,8 +5968,10 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 999 is opened
-Then the product page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/999) — on the catalogue, click product 999.
+4. On screen, verify: the product page reports not found.</t>
         </is>
       </c>
       <c r="H104" s="3" t="inlineStr">
@@ -6005,8 +6021,10 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 6 is opened
-Then the product page 6 is shown out of stock</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/6) — on the catalogue, click product 6.
+4. On screen, verify: the product page 6 is shown out of stock.</t>
         </is>
       </c>
       <c r="H105" s="3" t="inlineStr">
@@ -6056,9 +6074,11 @@
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 2 of product 1 and 1 of product 2
-When the order page is opened
-Then the order page total equals the stored order total</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): a placed order of 2 of product 1 and 1 of product 2.
+4. Open the app 'Order' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page total equals the stored order total.</t>
         </is>
       </c>
       <c r="H106" s="3" t="inlineStr">
@@ -6108,9 +6128,11 @@
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 1 of product 1
-When the order page is opened
-Then the order page shows the order id and status "placed"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): a placed order of 1 of product 1.
+4. Open the app 'Order' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page shows the order id and status "placed".</t>
         </is>
       </c>
       <c r="H107" s="3" t="inlineStr">
@@ -6160,7 +6182,9 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>Then every catalogue price is shown as a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: every catalogue price is shown as a dollar amount.</t>
         </is>
       </c>
       <c r="H108" s="3" t="inlineStr">
@@ -6210,7 +6234,9 @@
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue shows at least one product</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue shows at least one product.</t>
         </is>
       </c>
       <c r="H109" s="3" t="inlineStr">
@@ -6260,7 +6286,9 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>Then every catalogue name on screen equals the product row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: every catalogue name on screen equals the product row.</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr">
@@ -6310,8 +6338,10 @@
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>When the order page for 999999 is opened
-Then the order page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Order' screen in the browser (URL /order/999999) — open order 999999 from order history.
+4. On screen, verify: the order page reports not found.</t>
         </is>
       </c>
       <c r="H111" s="3" t="inlineStr">
@@ -6361,8 +6391,10 @@
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>When the product page for &lt;pid&gt; is opened
-Then the product page name, price and SKU equal row &lt;pid&gt;</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): the product page for &lt;pid&gt; is opened.
+4. On screen, verify: the product page name, price and SKU equal row &lt;pid&gt;.</t>
         </is>
       </c>
       <c r="H112" s="3" t="inlineStr">
@@ -6412,8 +6444,10 @@
       </c>
       <c r="G113" s="3" t="inlineStr">
         <is>
-          <t>When the product page for &lt;pid&gt; is opened
-Then the product page name, price and SKU equal row &lt;pid&gt;</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): the product page for &lt;pid&gt; is opened.
+4. On screen, verify: the product page name, price and SKU equal row &lt;pid&gt;.</t>
         </is>
       </c>
       <c r="H113" s="3" t="inlineStr">
@@ -6463,8 +6497,10 @@
       </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
-          <t>When the product page for &lt;pid&gt; is opened
-Then the product page name, price and SKU equal row &lt;pid&gt;</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): the product page for &lt;pid&gt; is opened.
+4. On screen, verify: the product page name, price and SKU equal row &lt;pid&gt;.</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr">
@@ -6514,7 +6550,9 @@
       </c>
       <c r="G115" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue price for product &lt;pid&gt; equals its row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue price for product &lt;pid&gt; equals its row.</t>
         </is>
       </c>
       <c r="H115" s="3" t="inlineStr">
@@ -6564,7 +6602,9 @@
       </c>
       <c r="G116" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue price for product &lt;pid&gt; equals its row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue price for product &lt;pid&gt; equals its row.</t>
         </is>
       </c>
       <c r="H116" s="3" t="inlineStr">
@@ -6614,7 +6654,9 @@
       </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue price for product &lt;pid&gt; equals its row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue price for product &lt;pid&gt; equals its row.</t>
         </is>
       </c>
       <c r="H117" s="3" t="inlineStr">
@@ -6664,7 +6706,9 @@
       </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
-          <t>Then the catalogue count equals the API active product count</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: the catalogue count equals the API active product count.</t>
         </is>
       </c>
       <c r="H118" s="3" t="inlineStr">
@@ -6714,8 +6758,10 @@
       </c>
       <c r="G119" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 3 is opened
-Then the product page price is shown as a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/3) — on the catalogue, click product 3.
+4. On screen, verify: the product page price is shown as a dollar amount.</t>
         </is>
       </c>
       <c r="H119" s="3" t="inlineStr">
@@ -6765,8 +6811,10 @@
       </c>
       <c r="G120" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 8 is opened
-Then the product page name is non-empty</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/8) — on the catalogue, click product 8.
+4. On screen, verify: the product page name is non-empty.</t>
         </is>
       </c>
       <c r="H120" s="3" t="inlineStr">
@@ -6816,9 +6864,11 @@
       </c>
       <c r="G121" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 1 of product 4
-When the order page is opened
-Then the order page total is shown as a dollar amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): a placed order of 1 of product 4.
+4. Open the app 'Order' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page total is shown as a dollar amount.</t>
         </is>
       </c>
       <c r="H121" s="3" t="inlineStr">
@@ -6868,7 +6918,9 @@
       </c>
       <c r="G122" s="3" t="inlineStr">
         <is>
-          <t>Then each catalogue row links to its product page</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: each catalogue row links to its product page.</t>
         </is>
       </c>
       <c r="H122" s="3" t="inlineStr">
@@ -6918,9 +6970,11 @@
       </c>
       <c r="G123" s="3" t="inlineStr">
         <is>
-          <t>Given a placed order of 2 of product 2 with coupon "SAVE10"
-When the order page is opened
-Then the order page total equals the stored order total</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Set up (before checking the screen): a placed order of 2 of product 2 with coupon "SAVE10".
+4. Open the app 'Order' screen in the browser (URL /order/&lt;the placed order&gt;) — click the placed order.
+5. On screen, verify: the order page total equals the stored order total.</t>
         </is>
       </c>
       <c r="H123" s="3" t="inlineStr">
@@ -6970,7 +7024,9 @@
       </c>
       <c r="G124" s="3" t="inlineStr">
         <is>
-          <t>Then every catalogue stock label is in stock or out of stock</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: every catalogue stock label is in stock or out of stock.</t>
         </is>
       </c>
       <c r="H124" s="3" t="inlineStr">
@@ -7020,8 +7076,10 @@
       </c>
       <c r="G125" s="3" t="inlineStr">
         <is>
-          <t>When the product page for 7 is opened
-Then the product page SKU equals row 7</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. Open the app 'Product' screen in the browser (URL /product/7) — on the catalogue, click product 7.
+4. On screen, verify: the product page SKU equals row 7.</t>
         </is>
       </c>
       <c r="H125" s="3" t="inlineStr">
@@ -7071,7 +7129,9 @@
       </c>
       <c r="G126" s="3" t="inlineStr">
         <is>
-          <t>Then no catalogue product id appears twice</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Set up (before checking the screen): the storefront is open.
+3. On screen, verify: no catalogue product id appears twice.</t>
         </is>
       </c>
       <c r="H126" s="3" t="inlineStr">
@@ -7121,7 +7181,8 @@
       </c>
       <c r="G127" s="3" t="inlineStr">
         <is>
-          <t>Then the number of products on screen equals the API product count</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the number of products on screen equals the API product count.</t>
         </is>
       </c>
       <c r="H127" s="3" t="inlineStr">
@@ -7171,7 +7232,8 @@
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>Then every product card on screen has a name and a price</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: every product card on screen has a name and a price.</t>
         </is>
       </c>
       <c r="H128" s="3" t="inlineStr">
@@ -7221,7 +7283,8 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Then every product price on screen matches the "Rs. N" format</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: every product price on screen matches the "Rs. N" format.</t>
         </is>
       </c>
       <c r="H129" s="3" t="inlineStr">
@@ -7271,7 +7334,8 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Then every product name on screen is in the API product list</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: every product name on screen is in the API product list.</t>
         </is>
       </c>
       <c r="H130" s="3" t="inlineStr">
@@ -7321,7 +7385,8 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Then the first product on screen matches the first API product</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the first product on screen matches the first API product.</t>
         </is>
       </c>
       <c r="H131" s="3" t="inlineStr">
@@ -7371,7 +7436,8 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>Then the screen shows at least 12 products</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the screen shows at least 12 products.</t>
         </is>
       </c>
       <c r="H132" s="3" t="inlineStr">
@@ -7421,7 +7487,8 @@
       </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
-          <t>Then no product card on screen is missing a price</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: no product card on screen is missing a price.</t>
         </is>
       </c>
       <c r="H133" s="3" t="inlineStr">
@@ -7471,7 +7538,8 @@
       </c>
       <c r="G134" s="3" t="inlineStr">
         <is>
-          <t>Then no product card on screen is missing a name</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: no product card on screen is missing a name.</t>
         </is>
       </c>
       <c r="H134" s="3" t="inlineStr">
@@ -7521,7 +7589,8 @@
       </c>
       <c r="G135" s="3" t="inlineStr">
         <is>
-          <t>Then the screen's product names are drawn from the API without inventing any</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the screen's product names are drawn from the API without inventing any.</t>
         </is>
       </c>
       <c r="H135" s="3" t="inlineStr">
@@ -7571,7 +7640,8 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t>Then every product price on screen parses to a non-negative number</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: every product price on screen parses to a non-negative number.</t>
         </is>
       </c>
       <c r="H136" s="3" t="inlineStr">
@@ -7621,8 +7691,9 @@
       </c>
       <c r="G137" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "Top"
-Then the search grid on screen is non-empty</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "Top".
+3. On screen, verify: the search grid on screen is non-empty.</t>
         </is>
       </c>
       <c r="H137" s="3" t="inlineStr">
@@ -7672,8 +7743,9 @@
       </c>
       <c r="G138" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "Dress"
-Then the search grid has no more products than the catalogue</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "Dress".
+3. On screen, verify: the search grid has no more products than the catalogue.</t>
         </is>
       </c>
       <c r="H138" s="3" t="inlineStr">
@@ -7723,8 +7795,9 @@
       </c>
       <c r="G139" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "Jeans"
-Then every search result name is in the API product list</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "Jeans".
+3. On screen, verify: every search result name is in the API product list.</t>
         </is>
       </c>
       <c r="H139" s="3" t="inlineStr">
@@ -7774,8 +7847,9 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "zzqqxx-no-such-product"
-Then the search grid on screen is empty</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "zzqqxx-no-such-product".
+3. On screen, verify: the search grid on screen is empty.</t>
         </is>
       </c>
       <c r="H140" s="3" t="inlineStr">
@@ -7825,8 +7899,9 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "Top"
-Then every product price on screen matches the "Rs. N" format</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "Top".
+3. On screen, verify: every product price on screen matches the "Rs. N" format.</t>
         </is>
       </c>
       <c r="H141" s="3" t="inlineStr">
@@ -7876,8 +7951,9 @@
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "&lt;term&gt;"
-Then the number of products on screen equals the API search count for "&lt;term&gt;"</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "&lt;term&gt;".
+3. On screen, verify: the number of products on screen equals the API search count for "&lt;term&gt;".</t>
         </is>
       </c>
       <c r="H142" s="3" t="inlineStr">
@@ -7927,8 +8003,9 @@
       </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "&lt;term&gt;"
-Then the number of products on screen equals the API search count for "&lt;term&gt;"</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "&lt;term&gt;".
+3. On screen, verify: the number of products on screen equals the API search count for "&lt;term&gt;".</t>
         </is>
       </c>
       <c r="H143" s="3" t="inlineStr">
@@ -7978,8 +8055,9 @@
       </c>
       <c r="G144" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "&lt;term&gt;"
-Then the number of products on screen equals the API search count for "&lt;term&gt;"</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "&lt;term&gt;".
+3. On screen, verify: the number of products on screen equals the API search count for "&lt;term&gt;".</t>
         </is>
       </c>
       <c r="H144" s="3" t="inlineStr">
@@ -8029,8 +8107,9 @@
       </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "top"
-Then the number of products on screen equals the API search count for "top"</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "top".
+3. On screen, verify: the number of products on screen equals the API search count for "top".</t>
         </is>
       </c>
       <c r="H145" s="3" t="inlineStr">
@@ -8080,8 +8159,9 @@
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t>When the brand rail is read
-Then every brand on screen is in the API brand list</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the brand rail is read.
+3. On screen, verify: every brand on screen is in the API brand list.</t>
         </is>
       </c>
       <c r="H146" s="3" t="inlineStr">
@@ -8131,8 +8211,9 @@
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
-          <t>When the brand rail is read
-Then the brand rail on screen is non-empty</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the brand rail is read.
+3. On screen, verify: the brand rail on screen is non-empty.</t>
         </is>
       </c>
       <c r="H147" s="3" t="inlineStr">
@@ -8182,8 +8263,9 @@
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t>When the brand rail is read
-Then no brand on screen is blank</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the brand rail is read.
+3. On screen, verify: no brand on screen is blank.</t>
         </is>
       </c>
       <c r="H148" s="3" t="inlineStr">
@@ -8233,7 +8315,8 @@
       </c>
       <c r="G149" s="3" t="inlineStr">
         <is>
-          <t>Then the product count on screen is the same on a second load</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the product count on screen is the same on a second load.</t>
         </is>
       </c>
       <c r="H149" s="3" t="inlineStr">
@@ -8283,7 +8366,8 @@
       </c>
       <c r="G150" s="3" t="inlineStr">
         <is>
-          <t>Then every product price on screen starts with "Rs."</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: every product price on screen starts with "Rs.".</t>
         </is>
       </c>
       <c r="H150" s="3" t="inlineStr">
@@ -8333,7 +8417,8 @@
       </c>
       <c r="G151" s="3" t="inlineStr">
         <is>
-          <t>Then every product name on screen is in the API product list</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: every product name on screen is in the API product list.</t>
         </is>
       </c>
       <c r="H151" s="3" t="inlineStr">
@@ -8383,7 +8468,8 @@
       </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
-          <t>Then the screen product names have no exact duplicates</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the screen product names have no exact duplicates.</t>
         </is>
       </c>
       <c r="H152" s="3" t="inlineStr">
@@ -8433,7 +8519,8 @@
       </c>
       <c r="G153" s="3" t="inlineStr">
         <is>
-          <t>Then the highest price on screen equals a price the API lists</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the highest price on screen equals a price the API lists.</t>
         </is>
       </c>
       <c r="H153" s="3" t="inlineStr">
@@ -8483,7 +8570,8 @@
       </c>
       <c r="G154" s="3" t="inlineStr">
         <is>
-          <t>Then the lowest price on screen equals a price the API lists</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the lowest price on screen equals a price the API lists.</t>
         </is>
       </c>
       <c r="H154" s="3" t="inlineStr">
@@ -8533,8 +8621,9 @@
       </c>
       <c r="G155" s="3" t="inlineStr">
         <is>
-          <t>When the storefront is searched for "Shirt"
-Then the search grid has no more products than the catalogue</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. Set up (before checking the screen): the storefront is searched for "Shirt".
+3. On screen, verify: the search grid has no more products than the catalogue.</t>
         </is>
       </c>
       <c r="H155" s="3" t="inlineStr">
@@ -8584,7 +8673,8 @@
       </c>
       <c r="G156" s="3" t="inlineStr">
         <is>
-          <t>Then the products page shows an "All Products" heading</t>
+          <t>1. Open the LIVE site 'Products storefront' screen in the browser (URL /products) — the products listing.
+2. On screen, verify: the products page shows an "All Products" heading.</t>
         </is>
       </c>
       <c r="H156" s="3" t="inlineStr">

</xml_diff>